<commit_message>
fix: rename NE/NE1/NE2/NE3 to EN/EN1/EN2/EN3 to avoid SPSS reserved word error
Agent-Logs-Url: https://github.com/via-zy/SEM-fsQCA/sessions/1d669677-dc07-468d-8689-4a9af03b65ee

Co-authored-by: via-zy <216556376+via-zy@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SEM_fsQCA_数据_已调整.xlsx
+++ b/SEM_fsQCA_数据_已调整.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数值数据" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="维度均值(fsQCA用)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变量说明" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人口统计学变量" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="数值数据" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="维度均值(fsQCA用)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="变量说明" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="人口统计学变量" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -506,17 +506,17 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>NE1</t>
+          <t>EN1</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>NE2</t>
+          <t>EN2</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>NE3</t>
+          <t>EN3</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
@@ -35126,7 +35126,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>EN</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -48492,7 +48492,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>EN</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -48502,7 +48502,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>NE1,NE2,NE3</t>
+          <t>EN1,EN2,EN3</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -48533,21 +48533,13 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>赋值标准</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -48560,8 +48552,6 @@
           <t>完全不认同=1, 不太认同=2, 一般=3, 比较认同=4, 完全认同=5</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix GP stats, add references [36]-[44], convert citations to [N] format, remove fake citations
Agent-Logs-Url: https://github.com/via-zy/SEM-fsQCA/sessions/16489e8f-7828-417a-a702-a62b0a586981

Co-authored-by: via-zy <216556376+via-zy@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SEM_fsQCA_数据_已调整.xlsx
+++ b/SEM_fsQCA_数据_已调整.xlsx
@@ -1001,8 +1001,6 @@
           <t>●</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1020,7 +1018,6 @@
           <t>●</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>●</t>
@@ -1038,8 +1035,6 @@
           <t>●</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>●</t>
@@ -1052,8 +1047,6 @@
           <t>TI（技术创新）</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>●</t>
@@ -1071,7 +1064,6 @@
           <t>DS（数字化能力）</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>●</t>
@@ -1082,7 +1074,6 @@
           <t>●</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1090,14 +1081,11 @@
           <t>EN（资源禀赋）</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3575,7 +3563,7 @@
         <v>5</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E36" t="n">
         <v>1</v>
@@ -4527,7 +4515,7 @@
         <v>4</v>
       </c>
       <c r="D50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E50" t="n">
         <v>2</v>
@@ -5547,7 +5535,7 @@
         <v>4</v>
       </c>
       <c r="D65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E65" t="n">
         <v>4</v>
@@ -9151,7 +9139,7 @@
         <v>5</v>
       </c>
       <c r="D118" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E118" t="n">
         <v>2</v>
@@ -10100,7 +10088,7 @@
         <v>3</v>
       </c>
       <c r="C132" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D132" t="n">
         <v>3</v>
@@ -12619,7 +12607,7 @@
         <v>4</v>
       </c>
       <c r="D169" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E169" t="n">
         <v>3</v>
@@ -13225,7 +13213,7 @@
         <v>177</v>
       </c>
       <c r="B178" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C178" t="n">
         <v>1</v>
@@ -13701,7 +13689,7 @@
         <v>184</v>
       </c>
       <c r="B185" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C185" t="n">
         <v>2</v>
@@ -13843,7 +13831,7 @@
         <v>5</v>
       </c>
       <c r="D187" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E187" t="n">
         <v>2</v>
@@ -14115,7 +14103,7 @@
         <v>5</v>
       </c>
       <c r="D191" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E191" t="n">
         <v>2</v>
@@ -15197,7 +15185,7 @@
         <v>206</v>
       </c>
       <c r="B207" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C207" t="n">
         <v>2</v>
@@ -17849,7 +17837,7 @@
         <v>245</v>
       </c>
       <c r="B246" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C246" t="n">
         <v>1</v>
@@ -18124,7 +18112,7 @@
         <v>3</v>
       </c>
       <c r="C250" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D250" t="n">
         <v>4</v>
@@ -18801,7 +18789,7 @@
         <v>259</v>
       </c>
       <c r="B260" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C260" t="n">
         <v>2</v>
@@ -19011,7 +18999,7 @@
         <v>5</v>
       </c>
       <c r="D263" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E263" t="n">
         <v>2</v>
@@ -19076,7 +19064,7 @@
         <v>3</v>
       </c>
       <c r="C264" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D264" t="n">
         <v>3</v>
@@ -19141,7 +19129,7 @@
         <v>264</v>
       </c>
       <c r="B265" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C265" t="n">
         <v>1</v>
@@ -20025,7 +20013,7 @@
         <v>277</v>
       </c>
       <c r="B278" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C278" t="n">
         <v>1</v>
@@ -20167,7 +20155,7 @@
         <v>5</v>
       </c>
       <c r="D280" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E280" t="n">
         <v>4</v>
@@ -21453,7 +21441,7 @@
         <v>298</v>
       </c>
       <c r="B299" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C299" t="n">
         <v>1</v>
@@ -21929,7 +21917,7 @@
         <v>305</v>
       </c>
       <c r="B306" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C306" t="n">
         <v>1</v>
@@ -22949,7 +22937,7 @@
         <v>320</v>
       </c>
       <c r="B321" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C321" t="n">
         <v>1</v>
@@ -23564,7 +23552,7 @@
         <v>3</v>
       </c>
       <c r="C330" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D330" t="n">
         <v>3</v>
@@ -24043,7 +24031,7 @@
         <v>4</v>
       </c>
       <c r="D337" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E337" t="n">
         <v>3</v>
@@ -24247,7 +24235,7 @@
         <v>5</v>
       </c>
       <c r="D340" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E340" t="n">
         <v>1</v>
@@ -24445,7 +24433,7 @@
         <v>342</v>
       </c>
       <c r="B343" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C343" t="n">
         <v>1</v>
@@ -24785,7 +24773,7 @@
         <v>347</v>
       </c>
       <c r="B348" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C348" t="n">
         <v>1</v>
@@ -25397,7 +25385,7 @@
         <v>356</v>
       </c>
       <c r="B357" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C357" t="n">
         <v>2</v>
@@ -26763,7 +26751,7 @@
         <v>4</v>
       </c>
       <c r="D377" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E377" t="n">
         <v>3</v>
@@ -27508,7 +27496,7 @@
         <v>2</v>
       </c>
       <c r="C388" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D388" t="n">
         <v>2</v>
@@ -29347,7 +29335,7 @@
         <v>3</v>
       </c>
       <c r="D415" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E415" t="n">
         <v>3</v>
@@ -29415,7 +29403,7 @@
         <v>5</v>
       </c>
       <c r="D416" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E416" t="n">
         <v>4</v>
@@ -30225,7 +30213,7 @@
         <v>427</v>
       </c>
       <c r="B428" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C428" t="n">
         <v>3</v>
@@ -30367,7 +30355,7 @@
         <v>5</v>
       </c>
       <c r="D430" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E430" t="n">
         <v>5</v>
@@ -31931,7 +31919,7 @@
         <v>3</v>
       </c>
       <c r="D453" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E453" t="n">
         <v>2</v>
@@ -32271,7 +32259,7 @@
         <v>3</v>
       </c>
       <c r="D458" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E458" t="n">
         <v>2</v>
@@ -34039,7 +34027,7 @@
         <v>4</v>
       </c>
       <c r="D484" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E484" t="n">
         <v>1</v>
@@ -34515,7 +34503,7 @@
         <v>3</v>
       </c>
       <c r="D491" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E491" t="n">
         <v>4</v>
@@ -34645,7 +34633,7 @@
         <v>492</v>
       </c>
       <c r="B493" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C493" t="n">
         <v>3</v>
@@ -35869,10 +35857,10 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>3</v>
+        <v>3.006</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.967</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>1</v>
@@ -35881,10 +35869,10 @@
         <v>5</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-0.028</v>
+        <v>-0.041</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-0.572</v>
+        <v>-0.657</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>508</v>
@@ -35900,7 +35888,7 @@
         <v>2.573</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.909</v>
+        <v>0.91</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>1</v>
@@ -35928,7 +35916,7 @@
         <v>3.321</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.949</v>
+        <v>0.95</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>1</v>
@@ -35956,7 +35944,7 @@
         <v>2.941</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>1</v>
@@ -36012,7 +36000,7 @@
         <v>3.636</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.908</v>
+        <v>0.909</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>1</v>
@@ -36040,7 +36028,7 @@
         <v>3.24</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>1</v>
@@ -36058,6 +36046,7 @@
         <v>508</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -36109,16 +36098,16 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>3</v>
+        <v>2.97</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>1.15</v>
+        <v>1.164</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0</v>
+        <v>0.057</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>-0.597</v>
+        <v>-0.68</v>
       </c>
     </row>
     <row r="13">
@@ -36133,16 +36122,16 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>3</v>
+        <v>3.01</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>1.15</v>
+        <v>1.147</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0</v>
+        <v>-0.019</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>-0.597</v>
+        <v>-0.5659999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -36157,16 +36146,16 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>3</v>
+        <v>3.037</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>1.15</v>
+        <v>1.167</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0</v>
+        <v>-0.073</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>-0.597</v>
+        <v>-0.699</v>
       </c>
     </row>
     <row r="15">
@@ -36184,7 +36173,7 @@
         <v>2.573</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1.126</v>
+        <v>1.127</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>0.298</v>
@@ -36208,7 +36197,7 @@
         <v>2.593</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>1.091</v>
+        <v>1.092</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>0.113</v>
@@ -36232,7 +36221,7 @@
         <v>2.555</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>1.111</v>
+        <v>1.112</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>0.244</v>
@@ -36256,7 +36245,7 @@
         <v>3.335</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>1.132</v>
+        <v>1.133</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>-0.234</v>
@@ -36280,7 +36269,7 @@
         <v>3.315</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>1.129</v>
+        <v>1.13</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>-0.156</v>
@@ -36304,7 +36293,7 @@
         <v>3.313</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1.166</v>
+        <v>1.168</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>-0.188</v>
@@ -36328,7 +36317,7 @@
         <v>2.937</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>1.157</v>
+        <v>1.158</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>0.016</v>
@@ -36352,7 +36341,7 @@
         <v>2.953</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>1.147</v>
+        <v>1.149</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>0.053</v>
@@ -36376,7 +36365,7 @@
         <v>2.933</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>1.141</v>
+        <v>1.142</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>0.012</v>
@@ -36400,7 +36389,7 @@
         <v>3.179</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>1.121</v>
+        <v>1.122</v>
       </c>
       <c r="E24" s="3" t="n">
         <v>-0.113</v>
@@ -36424,7 +36413,7 @@
         <v>3.177</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>1.14</v>
+        <v>1.141</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>-0.08699999999999999</v>
@@ -36448,7 +36437,7 @@
         <v>3.177</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>1.107</v>
+        <v>1.108</v>
       </c>
       <c r="E26" s="3" t="n">
         <v>-0.066</v>
@@ -36472,7 +36461,7 @@
         <v>3.648</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>1.096</v>
+        <v>1.097</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>-0.428</v>
@@ -36496,7 +36485,7 @@
         <v>3.608</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>1.097</v>
+        <v>1.098</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>-0.317</v>
@@ -36520,7 +36509,7 @@
         <v>3.652</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>1.118</v>
+        <v>1.119</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>-0.365</v>
@@ -36544,7 +36533,7 @@
         <v>3.23</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>1.114</v>
+        <v>1.115</v>
       </c>
       <c r="E30" s="3" t="n">
         <v>-0.06900000000000001</v>
@@ -36568,7 +36557,7 @@
         <v>3.232</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>1.157</v>
+        <v>1.159</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>-0.133</v>
@@ -36592,7 +36581,7 @@
         <v>3.258</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>1.134</v>
+        <v>1.135</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>-0.08799999999999999</v>

</xml_diff>